<commit_message>
fix: rewrite cuchara/cuchillo memory hook so both words make sense
The spreadsheet's hook for this confusing pair only explained
cuchillo (knife) — the cuchara (spoon) card was left with a tip
that never mentioned spoons. Rewrote the hook to lead with cuchara
and keep "LL = knife blades" as the contrast.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/spanish_english_cognates.xlsx
+++ b/data/spanish_english_cognates.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Formal English = Spanish" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Easy Associations" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Smart Hooks" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cognates by Pattern" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="False Friends (Watch Out)" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pattern Cheat Sheet" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Themed Cognates" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spanish for Spanish" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Formal English = Spanish" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Easy Associations" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Smart Hooks" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Cognates by Pattern" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="False Friends (Watch Out)" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Pattern Cheat Sheet" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Themed Cognates" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Spanish for Spanish" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -37380,7 +37380,7 @@
       </c>
       <c r="E89" s="41" t="inlineStr">
         <is>
-          <t>CuchiLLo = the two LL's look like knife blades standing up</t>
+          <t>Cuchara — no LL's, no blades, just a spoon. (CuchiLLo has two LL's like knife blades.)</t>
         </is>
       </c>
     </row>

</xml_diff>